<commit_message>
- Cambios en orden de archivos - Errores (en consola de momento)
</commit_message>
<xml_diff>
--- a/Carga_Real_FRAM Apply-Actualizado 28-11.xlsx
+++ b/Carga_Real_FRAM Apply-Actualizado 28-11.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7829" uniqueCount="1199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7830" uniqueCount="1200">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -2916,6 +2916,9 @@
   </si>
   <si>
     <t xml:space="preserve">P7849992B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-00</t>
   </si>
   <si>
     <t xml:space="preserve">RONNIE GIDOR</t>
@@ -28016,9 +28019,7 @@
       <c r="P2" s="110" t="s">
         <v>859</v>
       </c>
-      <c r="Q2" s="60" t="n">
-        <v>26176</v>
-      </c>
+      <c r="Q2" s="60"/>
       <c r="R2" s="43" t="s">
         <v>120</v>
       </c>
@@ -32355,8 +32356,8 @@
       <c r="BK22" s="9" t="n">
         <v>45614</v>
       </c>
-      <c r="BL22" s="115" t="n">
-        <v>0.416666666666667</v>
+      <c r="BL22" s="115" t="s">
+        <v>964</v>
       </c>
       <c r="BM22" s="61" t="s">
         <v>140</v>
@@ -32445,10 +32446,10 @@
         <v>106</v>
       </c>
       <c r="K23" s="110" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="M23" s="36" t="s">
         <v>150</v>
@@ -32460,7 +32461,7 @@
         <v>365</v>
       </c>
       <c r="P23" s="110" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="Q23" s="60" t="n">
         <v>27501</v>
@@ -32496,7 +32497,7 @@
         <v>955</v>
       </c>
       <c r="AB23" s="43" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="AC23" s="9" t="n">
         <v>45615</v>
@@ -32630,10 +32631,10 @@
         <v>106</v>
       </c>
       <c r="K24" s="110" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="M24" s="36" t="s">
         <v>150</v>
@@ -32645,7 +32646,7 @@
         <v>330</v>
       </c>
       <c r="P24" s="110" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="Q24" s="60" t="n">
         <v>29003</v>
@@ -32681,7 +32682,7 @@
         <v>922</v>
       </c>
       <c r="AB24" s="43" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="AC24" s="9" t="n">
         <v>45615</v>
@@ -32861,10 +32862,10 @@
         <v>106</v>
       </c>
       <c r="K25" s="110" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="M25" s="36" t="s">
         <v>150</v>
@@ -32876,7 +32877,7 @@
         <v>616</v>
       </c>
       <c r="P25" s="110" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="Q25" s="60" t="n">
         <v>29012</v>
@@ -33092,10 +33093,10 @@
         <v>106</v>
       </c>
       <c r="K26" s="110" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="M26" s="36" t="s">
         <v>150</v>
@@ -33107,7 +33108,7 @@
         <v>324</v>
       </c>
       <c r="P26" s="110" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="Q26" s="60" t="n">
         <v>30893</v>
@@ -33323,10 +33324,10 @@
         <v>106</v>
       </c>
       <c r="K27" s="110" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="M27" s="36" t="s">
         <v>150</v>
@@ -33338,7 +33339,7 @@
         <v>256</v>
       </c>
       <c r="P27" s="110" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="Q27" s="60" t="n">
         <v>32811</v>
@@ -33545,10 +33546,10 @@
         <v>106</v>
       </c>
       <c r="K28" s="110" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="L28" s="5" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="M28" s="36" t="s">
         <v>150</v>
@@ -33560,7 +33561,7 @@
         <v>338</v>
       </c>
       <c r="P28" s="110" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="Q28" s="60" t="n">
         <v>34913</v>
@@ -33593,7 +33594,7 @@
         <v>45616</v>
       </c>
       <c r="AA28" s="10" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="AB28" s="43" t="s">
         <v>956</v>
@@ -33767,10 +33768,10 @@
         <v>106</v>
       </c>
       <c r="K29" s="110" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="L29" s="5" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="M29" s="36" t="s">
         <v>150</v>
@@ -33782,7 +33783,7 @@
         <v>334</v>
       </c>
       <c r="P29" s="110" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="Q29" s="60" t="n">
         <v>34983</v>
@@ -33809,7 +33810,7 @@
         <v>869</v>
       </c>
       <c r="Y29" s="110" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="Z29" s="9" t="n">
         <v>45615</v>
@@ -33998,10 +33999,10 @@
         <v>106</v>
       </c>
       <c r="K30" s="110" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="M30" s="36" t="s">
         <v>150</v>
@@ -34010,10 +34011,10 @@
         <v>309</v>
       </c>
       <c r="O30" s="43" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="P30" s="110" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="Q30" s="60" t="n">
         <v>23895</v>
@@ -34046,7 +34047,7 @@
         <v>45615</v>
       </c>
       <c r="AA30" s="10" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="AB30" s="43" t="s">
         <v>956</v>
@@ -34232,10 +34233,10 @@
         <v>106</v>
       </c>
       <c r="K31" s="110" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="M31" s="36" t="s">
         <v>150</v>
@@ -34247,7 +34248,7 @@
         <v>373</v>
       </c>
       <c r="P31" s="110" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="Q31" s="60" t="n">
         <v>32270</v>
@@ -34274,13 +34275,13 @@
         <v>869</v>
       </c>
       <c r="Y31" s="110" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="Z31" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="AA31" s="10" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="AB31" s="43" t="s">
         <v>956</v>
@@ -34467,10 +34468,10 @@
         <v>106</v>
       </c>
       <c r="K32" s="110" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="L32" s="110" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="M32" s="36" t="s">
         <v>150</v>
@@ -34482,7 +34483,7 @@
         <v>359</v>
       </c>
       <c r="P32" s="110" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="Q32" s="60" t="n">
         <v>24881</v>
@@ -34509,7 +34510,7 @@
         <v>908</v>
       </c>
       <c r="Y32" s="110" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="Z32" s="9" t="n">
         <v>45616</v>
@@ -34617,10 +34618,10 @@
         <v>106</v>
       </c>
       <c r="K33" s="110" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="L33" s="110" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="M33" s="36" t="s">
         <v>150</v>
@@ -34632,7 +34633,7 @@
         <v>210</v>
       </c>
       <c r="P33" s="110" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="Q33" s="60" t="n">
         <v>32784</v>
@@ -34665,7 +34666,7 @@
         <v>45616</v>
       </c>
       <c r="AA33" s="10" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="AB33" s="43" t="s">
         <v>956</v>
@@ -34840,10 +34841,10 @@
         <v>106</v>
       </c>
       <c r="K34" s="110" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="L34" s="110" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="M34" s="36" t="s">
         <v>150</v>
@@ -34855,7 +34856,7 @@
         <v>379</v>
       </c>
       <c r="P34" s="110" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="Q34" s="60" t="n">
         <v>29907</v>
@@ -34875,7 +34876,7 @@
       <c r="V34" s="43"/>
       <c r="X34" s="123"/>
       <c r="Y34" s="110" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="Z34" s="124"/>
       <c r="AB34" s="43"/>
@@ -34955,10 +34956,10 @@
         <v>106</v>
       </c>
       <c r="K35" s="110" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="L35" s="110" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="M35" s="36" t="s">
         <v>114</v>
@@ -34970,7 +34971,7 @@
         <v>210</v>
       </c>
       <c r="P35" s="110" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="Q35" s="60" t="n">
         <v>25345</v>
@@ -35068,10 +35069,10 @@
         <v>106</v>
       </c>
       <c r="K36" s="110" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="L36" s="110" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="M36" s="36" t="s">
         <v>150</v>
@@ -35083,7 +35084,7 @@
         <v>227</v>
       </c>
       <c r="P36" s="110" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="Q36" s="60" t="n">
         <v>25862</v>
@@ -35185,7 +35186,7 @@
         <v>929</v>
       </c>
       <c r="L37" s="110" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="M37" s="36" t="s">
         <v>150</v>
@@ -35197,7 +35198,7 @@
         <v>151</v>
       </c>
       <c r="P37" s="110" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="Q37" s="60" t="n">
         <v>29694</v>
@@ -35295,10 +35296,10 @@
         <v>106</v>
       </c>
       <c r="K38" s="110" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="L38" s="110" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="M38" s="36" t="s">
         <v>114</v>
@@ -35310,7 +35311,7 @@
         <v>408</v>
       </c>
       <c r="P38" s="110" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="Q38" s="60" t="n">
         <v>26099</v>
@@ -35325,23 +35326,23 @@
         <v>120</v>
       </c>
       <c r="V38" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W38" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X38" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y38" s="110"/>
       <c r="Z38" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="AA38" s="10" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="AB38" s="43" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="AC38" s="4" t="n">
         <v>45616</v>
@@ -35436,10 +35437,10 @@
         <v>106</v>
       </c>
       <c r="K39" s="110" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="M39" s="36" t="s">
         <v>150</v>
@@ -35451,7 +35452,7 @@
         <v>548</v>
       </c>
       <c r="P39" s="110" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="Q39" s="60" t="n">
         <v>30878</v>
@@ -35466,16 +35467,16 @@
         <v>120</v>
       </c>
       <c r="V39" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W39" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X39" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y39" s="110" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="Z39" s="9" t="n">
         <v>45615</v>
@@ -35484,7 +35485,7 @@
         <v>936</v>
       </c>
       <c r="AB39" s="43" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="AC39" s="4" t="n">
         <v>45616</v>
@@ -35582,10 +35583,10 @@
         <v>106</v>
       </c>
       <c r="K40" s="110" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="M40" s="36" t="s">
         <v>150</v>
@@ -35597,7 +35598,7 @@
         <v>402</v>
       </c>
       <c r="P40" s="110" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="Q40" s="60" t="n">
         <v>30466</v>
@@ -35612,16 +35613,16 @@
         <v>120</v>
       </c>
       <c r="V40" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W40" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X40" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y40" s="110" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="Z40" s="9" t="n">
         <v>45615</v>
@@ -35630,7 +35631,7 @@
         <v>936</v>
       </c>
       <c r="AB40" s="43" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="AC40" s="4" t="n">
         <v>45616</v>
@@ -35728,22 +35729,22 @@
         <v>106</v>
       </c>
       <c r="K41" s="110" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="M41" s="36" t="s">
         <v>114</v>
       </c>
       <c r="N41" s="110" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="O41" s="110" t="s">
         <v>408</v>
       </c>
       <c r="P41" s="110" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="Q41" s="60" t="n">
         <v>35345</v>
@@ -35758,25 +35759,25 @@
         <v>120</v>
       </c>
       <c r="V41" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W41" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X41" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y41" s="110" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="Z41" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA41" s="10" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="AB41" s="43" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="AC41" s="4" t="n">
         <v>45616</v>
@@ -35901,22 +35902,22 @@
         <v>106</v>
       </c>
       <c r="K42" s="110" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="M42" s="36" t="s">
         <v>150</v>
       </c>
       <c r="N42" s="110" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="O42" s="110" t="s">
         <v>408</v>
       </c>
       <c r="P42" s="110" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="Q42" s="60" t="n">
         <v>25193</v>
@@ -35931,16 +35932,16 @@
         <v>120</v>
       </c>
       <c r="V42" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W42" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X42" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y42" s="110" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="Z42" s="9" t="n">
         <v>45616</v>
@@ -35949,7 +35950,7 @@
         <v>955</v>
       </c>
       <c r="AB42" s="43" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="AC42" s="4" t="n">
         <v>45617</v>
@@ -36074,22 +36075,22 @@
         <v>106</v>
       </c>
       <c r="K43" s="110" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="M43" s="36" t="s">
         <v>150</v>
       </c>
       <c r="N43" s="110" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="O43" s="110" t="s">
         <v>408</v>
       </c>
       <c r="P43" s="110" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="Q43" s="60" t="n">
         <v>21513</v>
@@ -36104,16 +36105,16 @@
         <v>120</v>
       </c>
       <c r="V43" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W43" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X43" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y43" s="110" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="Z43" s="9" t="n">
         <v>45616</v>
@@ -36122,7 +36123,7 @@
         <v>955</v>
       </c>
       <c r="AB43" s="43" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="AC43" s="4" t="n">
         <v>45617</v>
@@ -36247,10 +36248,10 @@
         <v>106</v>
       </c>
       <c r="K44" s="110" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="M44" s="36" t="s">
         <v>150</v>
@@ -36262,7 +36263,7 @@
         <v>239</v>
       </c>
       <c r="P44" s="110" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="Q44" s="60" t="n">
         <v>31770</v>
@@ -36277,16 +36278,16 @@
         <v>120</v>
       </c>
       <c r="V44" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W44" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X44" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y44" s="110" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="Z44" s="9" t="n">
         <v>45616</v>
@@ -36295,7 +36296,7 @@
         <v>909</v>
       </c>
       <c r="AB44" s="43" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="AC44" s="4" t="n">
         <v>45616</v>
@@ -36420,10 +36421,10 @@
         <v>106</v>
       </c>
       <c r="K45" s="110" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="M45" s="36" t="s">
         <v>150</v>
@@ -36435,7 +36436,7 @@
         <v>438</v>
       </c>
       <c r="P45" s="110" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="Q45" s="60" t="n">
         <v>34366</v>
@@ -36450,16 +36451,16 @@
         <v>120</v>
       </c>
       <c r="V45" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W45" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X45" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y45" s="110" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="Z45" s="9" t="n">
         <v>45616</v>
@@ -36468,7 +36469,7 @@
         <v>909</v>
       </c>
       <c r="AB45" s="43" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="AC45" s="4" t="n">
         <v>45616</v>
@@ -36593,10 +36594,10 @@
         <v>106</v>
       </c>
       <c r="K46" s="110" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="M46" s="36" t="s">
         <v>150</v>
@@ -36608,7 +36609,7 @@
         <v>425</v>
       </c>
       <c r="P46" s="110" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="Q46" s="60" t="n">
         <v>35627</v>
@@ -36623,25 +36624,25 @@
         <v>120</v>
       </c>
       <c r="V46" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W46" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X46" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y46" s="110" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="Z46" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA46" s="10" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="AB46" s="43" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="AC46" s="4" t="n">
         <v>45616</v>
@@ -36766,10 +36767,10 @@
         <v>106</v>
       </c>
       <c r="K47" s="110" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="M47" s="36" t="s">
         <v>150</v>
@@ -36781,7 +36782,7 @@
         <v>558</v>
       </c>
       <c r="P47" s="110" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="Q47" s="60" t="n">
         <v>36699</v>
@@ -36796,25 +36797,25 @@
         <v>120</v>
       </c>
       <c r="V47" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W47" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X47" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y47" s="110" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="Z47" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA47" s="10" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="AB47" s="43" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="AC47" s="4" t="n">
         <v>45616</v>
@@ -36939,22 +36940,22 @@
         <v>106</v>
       </c>
       <c r="K48" s="110" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="M48" s="36" t="s">
         <v>150</v>
       </c>
       <c r="N48" s="110" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="O48" s="110" t="s">
         <v>408</v>
       </c>
       <c r="P48" s="110" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="Q48" s="60" t="n">
         <v>33466</v>
@@ -36969,25 +36970,25 @@
         <v>120</v>
       </c>
       <c r="V48" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W48" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X48" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y48" s="110" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="Z48" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA48" s="10" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="AB48" s="43" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="AC48" s="4" t="n">
         <v>45616</v>
@@ -37112,10 +37113,10 @@
         <v>106</v>
       </c>
       <c r="K49" s="110" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="M49" s="36" t="s">
         <v>150</v>
@@ -37127,7 +37128,7 @@
         <v>455</v>
       </c>
       <c r="P49" s="110" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="Q49" s="60" t="n">
         <v>32481</v>
@@ -37142,25 +37143,25 @@
         <v>120</v>
       </c>
       <c r="V49" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W49" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X49" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y49" s="110" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="Z49" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA49" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="AB49" s="43" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="AC49" s="4" t="n">
         <v>45616</v>
@@ -37285,10 +37286,10 @@
         <v>106</v>
       </c>
       <c r="K50" s="110" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="M50" s="36" t="s">
         <v>150</v>
@@ -37300,7 +37301,7 @@
         <v>483</v>
       </c>
       <c r="P50" s="110" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="Q50" s="60" t="n">
         <v>33927</v>
@@ -37315,25 +37316,25 @@
         <v>120</v>
       </c>
       <c r="V50" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W50" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X50" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y50" s="110" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="Z50" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA50" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="AB50" s="43" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="AC50" s="4" t="n">
         <v>45616</v>
@@ -37458,10 +37459,10 @@
         <v>106</v>
       </c>
       <c r="K51" s="110" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="L51" s="5" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="M51" s="36" t="s">
         <v>114</v>
@@ -37473,7 +37474,7 @@
         <v>343</v>
       </c>
       <c r="P51" s="110" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="Q51" s="60" t="n">
         <v>32398</v>
@@ -37488,25 +37489,25 @@
         <v>120</v>
       </c>
       <c r="V51" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W51" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X51" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y51" s="110" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="Z51" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA51" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="AB51" s="43" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="AC51" s="4" t="n">
         <v>45616</v>
@@ -37631,10 +37632,10 @@
         <v>106</v>
       </c>
       <c r="K52" s="110" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="M52" s="36" t="s">
         <v>150</v>
@@ -37646,7 +37647,7 @@
         <v>334</v>
       </c>
       <c r="P52" s="110" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="Q52" s="60" t="n">
         <v>33314</v>
@@ -37661,25 +37662,25 @@
         <v>120</v>
       </c>
       <c r="V52" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W52" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X52" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y52" s="110" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="Z52" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA52" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="AB52" s="43" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="AC52" s="4" t="n">
         <v>45616</v>
@@ -37804,10 +37805,10 @@
         <v>106</v>
       </c>
       <c r="K53" s="110" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="L53" s="5" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="M53" s="36" t="s">
         <v>150</v>
@@ -37819,7 +37820,7 @@
         <v>210</v>
       </c>
       <c r="P53" s="110" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="Q53" s="60" t="n">
         <v>33838</v>
@@ -37834,25 +37835,25 @@
         <v>120</v>
       </c>
       <c r="V53" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W53" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X53" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y53" s="110" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="Z53" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA53" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="AB53" s="43" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="AC53" s="4" t="n">
         <v>45616</v>
@@ -37977,10 +37978,10 @@
         <v>106</v>
       </c>
       <c r="K54" s="110" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="M54" s="36" t="s">
         <v>150</v>
@@ -37992,7 +37993,7 @@
         <v>164</v>
       </c>
       <c r="P54" s="110" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="Q54" s="60" t="n">
         <v>27871</v>
@@ -38007,25 +38008,25 @@
         <v>120</v>
       </c>
       <c r="V54" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W54" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X54" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y54" s="110" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="Z54" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA54" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="AB54" s="43" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="AC54" s="4" t="n">
         <v>45616</v>
@@ -38150,22 +38151,22 @@
         <v>106</v>
       </c>
       <c r="K55" s="110" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="L55" s="5" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="M55" s="36" t="s">
         <v>114</v>
       </c>
       <c r="N55" s="110" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="O55" s="110" t="s">
         <v>571</v>
       </c>
       <c r="P55" s="110" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="Q55" s="60" t="n">
         <v>26518</v>
@@ -38180,25 +38181,25 @@
         <v>120</v>
       </c>
       <c r="V55" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W55" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X55" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y55" s="110" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="Z55" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA55" s="10" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="AB55" s="43" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="AC55" s="4" t="n">
         <v>45616</v>
@@ -38323,22 +38324,22 @@
         <v>106</v>
       </c>
       <c r="K56" s="110" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="M56" s="36" t="s">
         <v>114</v>
       </c>
       <c r="N56" s="110" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="O56" s="110" t="s">
         <v>402</v>
       </c>
       <c r="P56" s="110" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="Q56" s="60" t="n">
         <v>33209</v>
@@ -38353,25 +38354,25 @@
         <v>120</v>
       </c>
       <c r="V56" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W56" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X56" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y56" s="110" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="Z56" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA56" s="10" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="AB56" s="43" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="AC56" s="4" t="n">
         <v>45616</v>
@@ -38496,10 +38497,10 @@
         <v>106</v>
       </c>
       <c r="K57" s="110" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="M57" s="36" t="s">
         <v>150</v>
@@ -38511,7 +38512,7 @@
         <v>408</v>
       </c>
       <c r="P57" s="110" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="Q57" s="60" t="n">
         <v>33609</v>
@@ -38526,16 +38527,16 @@
         <v>540</v>
       </c>
       <c r="V57" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W57" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X57" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y57" s="110" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="Z57" s="9" t="n">
         <v>45615</v>
@@ -38544,7 +38545,7 @@
         <v>955</v>
       </c>
       <c r="AB57" s="43" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="AC57" s="4" t="n">
         <v>45616</v>
@@ -38638,10 +38639,10 @@
         <v>106</v>
       </c>
       <c r="K58" s="110" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="M58" s="36" t="s">
         <v>114</v>
@@ -38653,7 +38654,7 @@
         <v>448</v>
       </c>
       <c r="P58" s="110" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="Q58" s="60" t="n">
         <v>33431</v>
@@ -38668,16 +38669,16 @@
         <v>540</v>
       </c>
       <c r="V58" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W58" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X58" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y58" s="110" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="Z58" s="9" t="n">
         <v>45615</v>
@@ -38686,7 +38687,7 @@
         <v>955</v>
       </c>
       <c r="AB58" s="43" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="AC58" s="4" t="n">
         <v>45616</v>
@@ -38780,10 +38781,10 @@
         <v>106</v>
       </c>
       <c r="K59" s="110" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="M59" s="36" t="s">
         <v>114</v>
@@ -38795,7 +38796,7 @@
         <v>408</v>
       </c>
       <c r="P59" s="110" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="Q59" s="60" t="n">
         <v>34823</v>
@@ -38810,25 +38811,25 @@
         <v>120</v>
       </c>
       <c r="V59" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W59" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X59" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y59" s="110" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="Z59" s="9" t="n">
         <v>45616</v>
       </c>
       <c r="AA59" s="10" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="AB59" s="43" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="AC59" s="4" t="n">
         <v>45616</v>
@@ -38953,22 +38954,22 @@
         <v>106</v>
       </c>
       <c r="K60" s="110" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="L60" s="5" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="M60" s="36" t="s">
         <v>114</v>
       </c>
       <c r="N60" s="110" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="O60" s="110" t="s">
         <v>408</v>
       </c>
       <c r="P60" s="110" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="Q60" s="60" t="n">
         <v>23531</v>
@@ -38983,16 +38984,16 @@
         <v>600</v>
       </c>
       <c r="V60" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W60" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X60" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y60" s="110" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="Z60" s="9" t="n">
         <v>45615</v>
@@ -39001,7 +39002,7 @@
         <v>936</v>
       </c>
       <c r="AB60" s="43" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="AC60" s="4" t="n">
         <v>45616</v>
@@ -39043,7 +39044,7 @@
         <v>138</v>
       </c>
       <c r="AP60" s="10" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="BA60" s="61" t="s">
         <v>143</v>
@@ -39134,10 +39135,10 @@
         <v>106</v>
       </c>
       <c r="K61" s="130" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="L61" s="76" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="M61" s="49" t="s">
         <v>114</v>
@@ -39149,7 +39150,7 @@
         <v>708</v>
       </c>
       <c r="P61" s="130" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="Q61" s="129" t="n">
         <v>35127</v>
@@ -39164,13 +39165,13 @@
         <v>119</v>
       </c>
       <c r="V61" s="58" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W61" s="86" t="n">
         <v>45615</v>
       </c>
       <c r="X61" s="131" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y61" s="130" t="s">
         <v>941</v>
@@ -39182,7 +39183,7 @@
         <v>0.999305555555556</v>
       </c>
       <c r="AB61" s="58" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="AC61" s="77" t="n">
         <v>45616</v>
@@ -39293,10 +39294,10 @@
         <v>106</v>
       </c>
       <c r="K62" s="110" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="M62" s="36" t="s">
         <v>150</v>
@@ -39308,7 +39309,7 @@
         <v>294</v>
       </c>
       <c r="P62" s="110" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="Q62" s="60" t="n">
         <v>30583</v>
@@ -39323,16 +39324,16 @@
         <v>119</v>
       </c>
       <c r="V62" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W62" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X62" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y62" s="110" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="Z62" s="9" t="n">
         <v>45615</v>
@@ -39341,7 +39342,7 @@
         <v>950</v>
       </c>
       <c r="AB62" s="43" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="AC62" s="4" t="n">
         <v>45616</v>
@@ -39383,7 +39384,7 @@
         <v>138</v>
       </c>
       <c r="AP62" s="10" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="BA62" s="61" t="s">
         <v>143</v>
@@ -39475,10 +39476,10 @@
         <v>106</v>
       </c>
       <c r="K63" s="110" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="M63" s="36" t="s">
         <v>150</v>
@@ -39490,7 +39491,7 @@
         <v>116</v>
       </c>
       <c r="P63" s="110" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="Q63" s="60" t="n">
         <v>35635</v>
@@ -39505,16 +39506,16 @@
         <v>540</v>
       </c>
       <c r="V63" s="43" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="W63" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X63" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y63" s="110" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="Z63" s="9" t="n">
         <v>45616</v>
@@ -39604,7 +39605,7 @@
         <v>141</v>
       </c>
       <c r="BQ63" s="62" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="BR63" s="67" t="n">
         <v>0.916666666666667</v>
@@ -39645,10 +39646,10 @@
         <v>106</v>
       </c>
       <c r="K64" s="110" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="L64" s="5" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="M64" s="36" t="s">
         <v>150</v>
@@ -39657,10 +39658,10 @@
         <v>262</v>
       </c>
       <c r="O64" s="110" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="P64" s="110" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="Q64" s="60" t="n">
         <v>28169</v>
@@ -39675,13 +39676,13 @@
         <v>466</v>
       </c>
       <c r="V64" s="43" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="W64" s="9" t="n">
         <v>45615</v>
       </c>
       <c r="X64" s="7" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="Y64" s="110" t="s">
         <v>914</v>
@@ -39690,10 +39691,10 @@
         <v>45615</v>
       </c>
       <c r="AA64" s="10" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="AB64" s="43" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="AC64" s="4" t="n">
         <v>45616</v>
@@ -39809,22 +39810,22 @@
         <v>106</v>
       </c>
       <c r="K65" s="43" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="L65" s="10" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="M65" s="36" t="s">
         <v>150</v>
       </c>
       <c r="N65" s="110" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="O65" s="110" t="s">
         <v>779</v>
       </c>
       <c r="P65" s="110" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="Q65" s="9" t="n">
         <v>34570</v>
@@ -39839,31 +39840,31 @@
         <v>119</v>
       </c>
       <c r="V65" s="43" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W65" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X65" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y65" s="110" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="Z65" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="AA65" s="10" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="AB65" s="10" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="AC65" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD65" s="113" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="AE65" s="37" t="s">
         <v>132</v>
@@ -39950,10 +39951,10 @@
         <v>106</v>
       </c>
       <c r="K66" s="10" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="L66" s="10" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="M66" s="1" t="s">
         <v>150</v>
@@ -39980,31 +39981,31 @@
         <v>312</v>
       </c>
       <c r="V66" s="43" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W66" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X66" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y66" s="110" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="Z66" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="AA66" s="10" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="AB66" s="10" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="AC66" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD66" s="113" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="AE66" s="37" t="s">
         <v>132</v>
@@ -40095,22 +40096,22 @@
         <v>106</v>
       </c>
       <c r="K67" s="10" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="L67" s="10" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="M67" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N67" s="5" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="O67" s="5" t="s">
         <v>763</v>
       </c>
       <c r="P67" s="5" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="Q67" s="9" t="n">
         <v>33373</v>
@@ -40125,31 +40126,31 @@
         <v>119</v>
       </c>
       <c r="V67" s="43" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W67" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X67" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y67" s="110" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="Z67" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA67" s="10" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="AB67" s="10" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="AC67" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD67" s="113" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="AE67" s="37" t="s">
         <v>132</v>
@@ -40251,10 +40252,10 @@
         <v>106</v>
       </c>
       <c r="K68" s="10" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="L68" s="10" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="M68" s="1" t="s">
         <v>150</v>
@@ -40266,7 +40267,7 @@
         <v>425</v>
       </c>
       <c r="P68" s="5" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="Q68" s="9" t="n">
         <v>34881</v>
@@ -40281,31 +40282,31 @@
         <v>119</v>
       </c>
       <c r="V68" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W68" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X68" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y68" s="5" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="Z68" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA68" s="10" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="AB68" s="10" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="AC68" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD68" s="113" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="AE68" s="37" t="s">
         <v>132</v>
@@ -40410,22 +40411,22 @@
         <v>106</v>
       </c>
       <c r="K69" s="10" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="L69" s="10" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="M69" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N69" s="5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O69" s="5" t="s">
         <v>359</v>
       </c>
       <c r="P69" s="5" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="Q69" s="9" t="n">
         <v>33949</v>
@@ -40440,31 +40441,31 @@
         <v>119</v>
       </c>
       <c r="V69" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W69" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X69" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y69" s="5" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="Z69" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA69" s="10" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="AB69" s="10" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="AC69" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD69" s="113" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="AE69" s="37" t="s">
         <v>132</v>
@@ -40569,22 +40570,22 @@
         <v>106</v>
       </c>
       <c r="K70" s="10" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="L70" s="10" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="M70" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N70" s="5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O70" s="5" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="P70" s="5" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="Q70" s="9" t="n">
         <v>24371</v>
@@ -40599,31 +40600,31 @@
         <v>410</v>
       </c>
       <c r="V70" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W70" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X70" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y70" s="5" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="Z70" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA70" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="AB70" s="10" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="AC70" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD70" s="97" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="AE70" s="37" t="s">
         <v>132</v>
@@ -40728,22 +40729,22 @@
         <v>106</v>
       </c>
       <c r="K71" s="10" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="L71" s="10" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="M71" s="1" t="s">
         <v>114</v>
       </c>
       <c r="N71" s="5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O71" s="5" t="s">
         <v>834</v>
       </c>
       <c r="P71" s="5" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="Q71" s="9" t="n">
         <v>30318</v>
@@ -40758,31 +40759,31 @@
         <v>410</v>
       </c>
       <c r="V71" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W71" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X71" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y71" s="5" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="Z71" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA71" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="AB71" s="10" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="AC71" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD71" s="97" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="AE71" s="37" t="s">
         <v>132</v>
@@ -40887,22 +40888,22 @@
         <v>106</v>
       </c>
       <c r="K72" s="10" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="L72" s="10" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="M72" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O72" s="5" t="s">
         <v>717</v>
       </c>
       <c r="P72" s="5" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="Q72" s="9" t="n">
         <v>30106</v>
@@ -40917,31 +40918,31 @@
         <v>410</v>
       </c>
       <c r="V72" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W72" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X72" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y72" s="5" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="Z72" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA72" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="AB72" s="10" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="AC72" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD72" s="97" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="AE72" s="37" t="s">
         <v>132</v>
@@ -41046,22 +41047,22 @@
         <v>106</v>
       </c>
       <c r="K73" s="10" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="L73" s="10" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="M73" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N73" s="5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O73" s="5" t="s">
         <v>294</v>
       </c>
       <c r="P73" s="5" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="Q73" s="9" t="n">
         <v>31510</v>
@@ -41076,31 +41077,31 @@
         <v>410</v>
       </c>
       <c r="V73" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W73" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X73" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y73" s="5" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="Z73" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA73" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="AB73" s="10" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="AC73" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD73" s="97" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="AE73" s="37" t="s">
         <v>132</v>
@@ -41205,22 +41206,22 @@
         <v>106</v>
       </c>
       <c r="K74" s="10" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="L74" s="10" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="M74" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N74" s="5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O74" s="5" t="s">
         <v>730</v>
       </c>
       <c r="P74" s="5" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="Q74" s="9" t="n">
         <v>26595</v>
@@ -41235,31 +41236,31 @@
         <v>410</v>
       </c>
       <c r="V74" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W74" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X74" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y74" s="5" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="Z74" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA74" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="AB74" s="10" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="AC74" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD74" s="97" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="AE74" s="37" t="s">
         <v>132</v>
@@ -41364,16 +41365,16 @@
         <v>106</v>
       </c>
       <c r="K75" s="10" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="L75" s="10" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="M75" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N75" s="5" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="O75" s="5" t="s">
         <v>786</v>
@@ -41394,31 +41395,31 @@
         <v>312</v>
       </c>
       <c r="V75" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W75" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X75" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y75" s="5" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="Z75" s="9" t="n">
         <v>45626</v>
       </c>
       <c r="AA75" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="AB75" s="10" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="AC75" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD75" s="97" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="AE75" s="37" t="s">
         <v>132</v>
@@ -41454,7 +41455,7 @@
         <v>176</v>
       </c>
       <c r="AP75" s="10" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="BA75" s="1" t="s">
         <v>143</v>
@@ -41523,10 +41524,10 @@
         <v>106</v>
       </c>
       <c r="K76" s="10" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="L76" s="10" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="M76" s="1" t="s">
         <v>150</v>
@@ -41538,7 +41539,7 @@
         <v>116</v>
       </c>
       <c r="P76" s="5" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="Q76" s="9" t="n">
         <v>34906</v>
@@ -41553,7 +41554,7 @@
         <v>119</v>
       </c>
       <c r="V76" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W76" s="9" t="n">
         <v>45625</v>
@@ -41568,7 +41569,7 @@
         <v>45626</v>
       </c>
       <c r="AA76" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="AB76" s="10" t="s">
         <v>932</v>
@@ -41577,7 +41578,7 @@
         <v>45626</v>
       </c>
       <c r="AD76" s="97" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="AE76" s="37" t="s">
         <v>132</v>
@@ -41679,22 +41680,22 @@
         <v>106</v>
       </c>
       <c r="K77" s="10" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="L77" s="10" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="M77" s="1" t="s">
         <v>150</v>
       </c>
       <c r="N77" s="5" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="O77" s="5" t="s">
         <v>812</v>
       </c>
       <c r="P77" s="5" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="Q77" s="9" t="n">
         <v>34260</v>
@@ -41709,31 +41710,31 @@
         <v>119</v>
       </c>
       <c r="V77" s="10" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="W77" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="X77" s="5" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="Y77" s="5" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="Z77" s="9" t="n">
         <v>45625</v>
       </c>
       <c r="AA77" s="10" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="AB77" s="10" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="AC77" s="4" t="n">
         <v>45626</v>
       </c>
       <c r="AD77" s="97" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="AE77" s="37" t="s">
         <v>132</v>

</xml_diff>

<commit_message>
Arreglado escalado infinito de botones. Creado archivo utils.py
</commit_message>
<xml_diff>
--- a/Carga_Real_FRAM Apply-Actualizado 28-11.xlsx
+++ b/Carga_Real_FRAM Apply-Actualizado 28-11.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7817" uniqueCount="1199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7816" uniqueCount="1199">
   <si>
     <t xml:space="preserve">Activo</t>
   </si>
@@ -13586,8 +13586,8 @@
       <c r="AI38" s="38" t="n">
         <v>45610</v>
       </c>
-      <c r="AJ38" s="41" t="s">
-        <v>235</v>
+      <c r="AJ38" s="41" t="n">
+        <v>0.597222222222222</v>
       </c>
       <c r="AK38" s="44" t="s">
         <v>305</v>

</xml_diff>